<commit_message>
Update buybacks to $750M/yr across model, financials, and slides
- Raise fixed repurchase assumption from $500M to $750M in 3-statement,
  DCF Scenarios (bb_fixed), and repurchase schedule
- Recompute forecast EPS, share retirement (32.9M), and cash roll-forward
- Update Risk & Mitigants and Timeline slides with $750M buyback references
- Refresh pitch_values.json and rebuild deck/PDF

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULUMODEL18.xlsx
+++ b/LULU/LULUMODEL18.xlsx
@@ -2644,10 +2644,10 @@
         </is>
       </c>
       <c r="F21" s="37" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="G21" s="37" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="H21" s="37" t="n">
         <v>0</v>
@@ -11634,7 +11634,7 @@
         </is>
       </c>
       <c r="E65" s="37" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="F65" s="37">
         <f>$E$65</f>

</xml_diff>

<commit_message>
Remove Firecrawl and agent references from model18altered build scripts
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULUMODEL18.xlsx
+++ b/LULU/LULUMODEL18.xlsx
@@ -5847,7 +5847,7 @@
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>FY2025A = Firecrawl-ingested 10-K anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
+          <t>FY2025A = sourced 10-K anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>Phases 1–4 clean and forecast operating profit; Phase 5 is the agent workflow summary below.</t>
+          <t>Phases 1–4 clean and forecast operating profit; Phase 5 summarizes the reconciliation workflow below.</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
     <row r="43">
       <c r="A43" s="73" t="inlineStr">
         <is>
-          <t>Phase 5 — Agent workflow (execution steps)</t>
+          <t>Phase 5 — Reconciliation workflow (execution steps)</t>
         </is>
       </c>
     </row>
@@ -13120,7 +13120,7 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ALO YOGA BUILD — no source prints EV/EBITDA (Firecrawl: Reuters + Forbes)</t>
+          <t>ALO YOGA BUILD — no source prints EV/EBITDA (Reuters + Forbes)</t>
         </is>
       </c>
     </row>
@@ -13202,7 +13202,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
+          <t>No Ctrl+F for EV/EBITDA — none found on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
       <c r="E35" s="118">

</xml_diff>